<commit_message>
update TEST EXECUTION logout 1
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40AF8AC6-3607-4D6B-8BDE-415EDC62CC77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC03177-9273-44D6-A21D-C6941CE75AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
   <sheets>
     <sheet name="EXE Regisration " sheetId="1" r:id="rId1"/>
     <sheet name="EXE Login" sheetId="2" r:id="rId2"/>
     <sheet name="EXE Authorization" sheetId="3" r:id="rId3"/>
     <sheet name="EXE Logout" sheetId="4" r:id="rId4"/>
+    <sheet name="EXE Session" sheetId="5" r:id="rId5"/>
+    <sheet name="EXE UI" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="102">
   <si>
     <t>SUB</t>
   </si>
@@ -334,6 +336,15 @@
   </si>
   <si>
     <t>User cannot access restricted paage after logout</t>
+  </si>
+  <si>
+    <t>Session Module</t>
+  </si>
+  <si>
+    <t>Verify session is active after successful login</t>
+  </si>
+  <si>
+    <t>Verify error message is clearly visible to the user</t>
   </si>
 </sst>
 </file>
@@ -497,22 +508,22 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1024,10 +1035,10 @@
       </c>
     </row>
     <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1068,8 +1079,8 @@
       </c>
     </row>
     <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="12"/>
-      <c r="E9" s="15"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1108,10 +1119,10 @@
       </c>
     </row>
     <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>55</v>
       </c>
       <c r="F10" s="4" t="s">
@@ -1152,8 +1163,8 @@
       </c>
     </row>
     <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D11" s="12"/>
-      <c r="E11" s="15"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="4" t="s">
         <v>53</v>
       </c>
@@ -1444,10 +1455,10 @@
       </c>
     </row>
     <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1488,8 +1499,8 @@
       </c>
     </row>
     <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="11"/>
-      <c r="E9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1528,8 +1539,8 @@
       </c>
     </row>
     <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="12"/>
-      <c r="E10" s="15"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4" t="s">
         <v>61</v>
       </c>
@@ -1818,10 +1829,10 @@
       </c>
     </row>
     <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1862,8 +1873,8 @@
       </c>
     </row>
     <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="11"/>
-      <c r="E9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1902,8 +1913,8 @@
       </c>
     </row>
     <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="12"/>
-      <c r="E10" s="15"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="4" t="s">
         <v>61</v>
       </c>
@@ -2081,7 +2092,7 @@
         <v>91</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>22</v>
@@ -2195,4 +2206,408 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5865AA9-EF4D-4605-AE01-BF23E8F15ED8}">
+  <dimension ref="D4:Q11"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="6"/>
+    <col min="4" max="4" width="8.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:17" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="4:17" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P5" s="7">
+        <v>46080</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P6" s="7">
+        <v>46080</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P7" s="7">
+        <v>46081</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94E22900-4FE0-414D-8528-401B4B671706}">
+  <dimension ref="D4:Q11"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="6"/>
+    <col min="4" max="4" width="8.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="4:17" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="4:17" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P5" s="7">
+        <v>46080</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P6" s="7">
+        <v>46080</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="D7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="P7" s="7">
+        <v>46081</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update TEST EXECUTION session 1
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC03177-9273-44D6-A21D-C6941CE75AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1412B7C-CB5B-4EE6-A678-907149A4A0B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
   <sheets>
     <sheet name="EXE Regisration " sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="103">
   <si>
     <t>SUB</t>
   </si>
@@ -345,6 +345,9 @@
   </si>
   <si>
     <t>Verify error message is clearly visible to the user</t>
+  </si>
+  <si>
+    <t>User successfully logged in without relogin</t>
   </si>
 </sst>
 </file>
@@ -2295,7 +2298,7 @@
         <v>91</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
upload TEST EXECUTION session 3
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156E11F4-9889-4406-9653-05D1B430A076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6818813A-27CF-4EC8-AC3B-C1CB160BD7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="108">
   <si>
     <t>SUB</t>
   </si>
@@ -354,6 +354,17 @@
   </si>
   <si>
     <t>User successful logged in</t>
+  </si>
+  <si>
+    <t>Verify restricted page cannot be accessed 
+using browser back button after logout</t>
+  </si>
+  <si>
+    <t>Verify restricted page cannot be accessed 
+via browser back after logout</t>
+  </si>
+  <si>
+    <t>User cannot access restricted page after logout then click back button</t>
   </si>
 </sst>
 </file>
@@ -490,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -534,6 +545,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2230,7 +2244,7 @@
     <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="62.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" style="6" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
@@ -2373,26 +2387,26 @@
       <c r="D7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>96</v>
+      <c r="E7" s="16" t="s">
+        <v>105</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>35</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>97</v>
+      <c r="I7" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>94</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>22</v>
@@ -2407,7 +2421,7 @@
         <v>20</v>
       </c>
       <c r="P7" s="7">
-        <v>46081</v>
+        <v>46086</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
upload TEST EXECUTION UI 1
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6818813A-27CF-4EC8-AC3B-C1CB160BD7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F06D1D-043A-4966-AF1B-80C145898C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
   <sheets>
     <sheet name="EXE Regisration " sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="111">
   <si>
     <t>SUB</t>
   </si>
@@ -365,6 +365,15 @@
   </si>
   <si>
     <t>User cannot access restricted page after logout then click back button</t>
+  </si>
+  <si>
+    <t>UI Module</t>
+  </si>
+  <si>
+    <t>Error message is clearly visible, readable, and positioned near related field</t>
+  </si>
+  <si>
+    <t>Error message appears clearly to user</t>
   </si>
 </sst>
 </file>
@@ -2444,11 +2453,11 @@
     <col min="6" max="6" width="12.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="37.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" style="6" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="9.140625" style="6"/>
   </cols>
@@ -2508,19 +2517,19 @@
         <v>11</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>91</v>
+      <c r="I5" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>22</v>
@@ -2535,7 +2544,7 @@
         <v>20</v>
       </c>
       <c r="P5" s="7">
-        <v>46080</v>
+        <v>46086</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>21</v>
@@ -2579,7 +2588,7 @@
         <v>20</v>
       </c>
       <c r="P6" s="7">
-        <v>46080</v>
+        <v>46086</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>26</v>
@@ -2623,7 +2632,7 @@
         <v>20</v>
       </c>
       <c r="P7" s="7">
-        <v>46081</v>
+        <v>46086</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
upload TEST EXECUTION UI 2
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F06D1D-043A-4966-AF1B-80C145898C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AE47B6-BA0C-4AB8-B41E-B920A572E922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="115">
   <si>
     <t>SUB</t>
   </si>
@@ -374,6 +374,19 @@
   </si>
   <si>
     <t>Error message appears clearly to user</t>
+  </si>
+  <si>
+    <t>Verify form validation appears when input is incorrect</t>
+  </si>
+  <si>
+    <t>Verify validation message for
+ incorrect input</t>
+  </si>
+  <si>
+    <t>Validation message appears for each incorrect field</t>
+  </si>
+  <si>
+    <t>Error message appears clearly to user in filed  who has incorrect and invalid format</t>
   </si>
 </sst>
 </file>
@@ -2555,25 +2568,25 @@
         <v>24</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>93</v>
+      <c r="I6" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>22</v>
@@ -2605,7 +2618,7 @@
         <v>35</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
upload TEST EXECUTION UI 3
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AE47B6-BA0C-4AB8-B41E-B920A572E922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9C8BFC-6CEF-436E-A89C-F683C88B8371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="119">
   <si>
     <t>SUB</t>
   </si>
@@ -387,6 +387,18 @@
   </si>
   <si>
     <t>Error message appears clearly to user in filed  who has incorrect and invalid format</t>
+  </si>
+  <si>
+    <t>Verify system display is responsive on mobile devices</t>
+  </si>
+  <si>
+    <t>Verify system responsiveness on mobile view</t>
+  </si>
+  <si>
+    <t>Layout adjusts properly, no overlapping text/buttons, all features accessible</t>
+  </si>
+  <si>
+    <t>Layout work properly on all devices include mobile</t>
   </si>
 </sst>
 </file>
@@ -2468,7 +2480,7 @@
     <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="43.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="37.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="74" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" style="6" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
@@ -2611,8 +2623,8 @@
       <c r="D7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>96</v>
+      <c r="E7" s="16" t="s">
+        <v>115</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>35</v>
@@ -2623,14 +2635,14 @@
       <c r="H7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>97</v>
+      <c r="I7" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
update TEST EXECUTION Authorization 1
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9C8BFC-6CEF-436E-A89C-F683C88B8371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9144E51E-AD4E-40DB-B74D-F0B67742AB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
   <sheets>
     <sheet name="EXE Regisration " sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="124">
   <si>
     <t>SUB</t>
   </si>
@@ -399,6 +399,22 @@
   </si>
   <si>
     <t>Layout work properly on all devices include mobile</t>
+  </si>
+  <si>
+    <t>Verify redirect to login when accessing
+ restricted page via direct URL</t>
+  </si>
+  <si>
+    <t>Verify user cannot access restricted page without login</t>
+  </si>
+  <si>
+    <t>Verify logged-in user can access restricted page</t>
+  </si>
+  <si>
+    <t>Authorization Module</t>
+  </si>
+  <si>
+    <t>Access restricted page without login</t>
   </si>
 </sst>
 </file>
@@ -562,6 +578,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -579,9 +598,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1092,10 +1108,10 @@
       </c>
     </row>
     <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>44</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1136,8 +1152,8 @@
       </c>
     </row>
     <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="13"/>
-      <c r="E9" s="11"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="12"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1176,10 +1192,10 @@
       </c>
     </row>
     <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>55</v>
       </c>
       <c r="F10" s="4" t="s">
@@ -1220,8 +1236,8 @@
       </c>
     </row>
     <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D11" s="13"/>
-      <c r="E11" s="11"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="12"/>
       <c r="F11" s="4" t="s">
         <v>53</v>
       </c>
@@ -1512,10 +1528,10 @@
       </c>
     </row>
     <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>80</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -1556,8 +1572,8 @@
       </c>
     </row>
     <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="16"/>
       <c r="F9" s="4" t="s">
         <v>48</v>
       </c>
@@ -1596,8 +1612,8 @@
       </c>
     </row>
     <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="13"/>
-      <c r="E10" s="11"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="12"/>
       <c r="F10" s="4" t="s">
         <v>61</v>
       </c>
@@ -1698,13 +1714,13 @@
     <col min="4" max="4" width="8.42578125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" style="6" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21" style="6" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="9.140625" style="6"/>
   </cols>
@@ -1758,25 +1774,25 @@
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>22</v>
@@ -1791,7 +1807,7 @@
         <v>20</v>
       </c>
       <c r="P5" s="7">
-        <v>46077</v>
+        <v>46086</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>21</v>
@@ -1801,14 +1817,14 @@
       <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>72</v>
+      <c r="E6" s="10" t="s">
+        <v>119</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>24</v>
@@ -1835,7 +1851,7 @@
         <v>20</v>
       </c>
       <c r="P6" s="7">
-        <v>46077</v>
+        <v>46086</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>26</v>
@@ -1845,14 +1861,14 @@
       <c r="D7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>76</v>
+      <c r="E7" s="10" t="s">
+        <v>121</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>35</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>34</v>
@@ -1879,185 +1895,14 @@
         <v>20</v>
       </c>
       <c r="P7" s="7">
-        <v>46077</v>
+        <v>46086</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D8" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="P8" s="7">
-        <v>46077</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N9" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="P9" s="7">
-        <v>46077</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D10" s="13"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="P10" s="7">
-        <v>46077</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="D11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="P11" s="7">
-        <v>46078</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
+    <row r="11" spans="4:17" ht="31.5" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2421,7 +2266,7 @@
       <c r="D7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="10" t="s">
         <v>105</v>
       </c>
       <c r="F7" s="4" t="s">
@@ -2623,7 +2468,7 @@
       <c r="D7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="10" t="s">
         <v>115</v>
       </c>
       <c r="F7" s="4" t="s">

</xml_diff>

<commit_message>
update TEST EXECUTION Authorization 2
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9144E51E-AD4E-40DB-B74D-F0B67742AB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10CB2AE8-AC94-41BF-8CDD-954C1F04D09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="127">
   <si>
     <t>SUB</t>
   </si>
@@ -415,6 +415,17 @@
   </si>
   <si>
     <t>Access restricted page without login</t>
+  </si>
+  <si>
+    <t>Access restricted page via direct 
+URL without login</t>
+  </si>
+  <si>
+    <t>User cannot access restricted page and direct to 
+register / login page</t>
+  </si>
+  <si>
+    <t>User redirected to register / login page</t>
   </si>
 </sst>
 </file>
@@ -1717,7 +1728,7 @@
     <col min="7" max="7" width="20" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="41.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="43.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="58.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="15" width="21" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11" style="6" bestFit="1" customWidth="1"/>
@@ -1829,14 +1840,14 @@
       <c r="H6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>29</v>
+      <c r="I6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
update TEST EXECUTION Authorization 3
</commit_message>
<xml_diff>
--- a/documentation/TEST EXECUTION.xlsx
+++ b/documentation/TEST EXECUTION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Worpdress Blog Manual Testing\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10CB2AE8-AC94-41BF-8CDD-954C1F04D09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4FAF98-E33B-4BCB-AA9E-37D519DA28AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{1DDAD4FE-2D96-4A5D-8208-8609A00B936D}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="130">
   <si>
     <t>SUB</t>
   </si>
@@ -426,6 +426,15 @@
   </si>
   <si>
     <t>User redirected to register / login page</t>
+  </si>
+  <si>
+    <t>Access restricted page after login</t>
+  </si>
+  <si>
+    <t>User can access restricted page</t>
+  </si>
+  <si>
+    <t>Restricted page successful apears on user who login on the system</t>
   </si>
 </sst>
 </file>
@@ -1884,23 +1893,23 @@
       <c r="H7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>77</v>
+      <c r="I7" s="5" t="s">
+        <v>127</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>31</v>
+        <v>129</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>22</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="O7" s="4" t="s">
         <v>20</v>

</xml_diff>